<commit_message>
ajout parcelle Bousquet et Riou
</commit_message>
<xml_diff>
--- a/irrigation_truffiere_2026.xlsx
+++ b/irrigation_truffiere_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="1" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="1" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Paramètres &amp; ETc" sheetId="1" state="hidden" r:id="rId3"/>
@@ -14,7 +14,8 @@
     <sheet name="Piles" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="La Fontaine" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="La baume" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Modèle saisie" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Bousquet et Riou" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Modèle saisie" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="124">
   <si>
     <t xml:space="preserve">CALENDRIER D'IRRIGATION TRUFFIÈRE — SAISON MAI–SEPTEMBRE 2026</t>
   </si>
@@ -436,7 +437,16 @@
     <t xml:space="preserve">mm</t>
   </si>
   <si>
+    <t xml:space="preserve">TOTAL Juin</t>
+  </si>
+  <si>
     <t xml:space="preserve">Durée d’arrosage (h)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ligne 1 Bousquet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ligne 2 Riou</t>
   </si>
 </sst>
 </file>
@@ -1017,7 +1027,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="144">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1422,6 +1432,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1430,10 +1444,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="0" fillId="21" borderId="13" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1463,6 +1473,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="22" borderId="17" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1662,34 +1684,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -3714,11 +3736,13 @@
         <v>119</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="13.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" s="101" customFormat="true" ht="13.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="73"/>
       <c r="B16" s="73"/>
       <c r="C16" s="73"/>
       <c r="D16" s="73"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="92" t="n">
         <v>46198</v>
       </c>
@@ -3729,11 +3753,15 @@
         <f aca="false">(H16/C2)/10</f>
         <v>17.4216027874564</v>
       </c>
-      <c r="J16" s="95"/>
-      <c r="K16" s="96"/>
+      <c r="J16" s="95" t="n">
+        <v>46202</v>
+      </c>
+      <c r="K16" s="96" t="n">
+        <v>366</v>
+      </c>
       <c r="L16" s="97" t="n">
         <f aca="false">(K16/C3)/10</f>
-        <v>0</v>
+        <v>21.6953171310018</v>
       </c>
       <c r="M16" s="98" t="n">
         <v>46199</v>
@@ -3747,11 +3775,13 @@
         <v>54.6875</v>
       </c>
     </row>
-    <row r="17" s="103" customFormat="true" ht="13.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
+    <row r="17" customFormat="false" ht="13.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="102"/>
+      <c r="B17" s="103"/>
+      <c r="C17" s="103"/>
+      <c r="D17" s="103"/>
+      <c r="E17" s="101"/>
+      <c r="F17" s="101"/>
       <c r="G17" s="104" t="n">
         <v>46200</v>
       </c>
@@ -3774,34 +3804,45 @@
       <c r="B18" s="70"/>
       <c r="C18" s="70"/>
       <c r="D18" s="70"/>
-      <c r="G18" s="104"/>
-      <c r="H18" s="105" t="n">
-        <f aca="false">H17</f>
-        <v>474.428571428571</v>
-      </c>
-      <c r="I18" s="94" t="n">
-        <f aca="false">(H18/C2)/10</f>
-        <v>27.5510204081633</v>
-      </c>
-      <c r="J18" s="106"/>
-      <c r="K18" s="107"/>
-      <c r="L18" s="108"/>
-      <c r="M18" s="109"/>
-      <c r="N18" s="110"/>
-      <c r="O18" s="111"/>
+      <c r="G18" s="112" t="s">
+        <v>120</v>
+      </c>
+      <c r="H18" s="113" t="n">
+        <f aca="false">SUM(H16:H17)</f>
+        <v>774.428571428571</v>
+      </c>
+      <c r="I18" s="114" t="n">
+        <f aca="false">SUM(I16:I17)</f>
+        <v>44.9726231956197</v>
+      </c>
+      <c r="J18" s="114"/>
+      <c r="K18" s="114" t="n">
+        <f aca="false">SUM(K16:K17)</f>
+        <v>366</v>
+      </c>
+      <c r="L18" s="114" t="n">
+        <f aca="false">SUM(L16:L17)</f>
+        <v>21.6953171310018</v>
+      </c>
+      <c r="M18" s="114"/>
+      <c r="N18" s="114" t="n">
+        <f aca="false">SUM(N16:N17)</f>
+        <v>280</v>
+      </c>
+      <c r="O18" s="114" t="n">
+        <f aca="false">SUM(O16:O17)</f>
+        <v>54.6875</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="70"/>
       <c r="C19" s="70"/>
       <c r="D19" s="70"/>
       <c r="G19" s="104"/>
-      <c r="H19" s="105" t="n">
-        <f aca="false">H18</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H19" s="105"/>
       <c r="I19" s="94" t="n">
         <f aca="false">(H19/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J19" s="106"/>
       <c r="K19" s="107"/>
@@ -3815,13 +3856,10 @@
       <c r="C20" s="70"/>
       <c r="D20" s="70"/>
       <c r="G20" s="104"/>
-      <c r="H20" s="105" t="n">
-        <f aca="false">H19</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H20" s="105"/>
       <c r="I20" s="94" t="n">
         <f aca="false">(H20/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J20" s="106"/>
       <c r="K20" s="107"/>
@@ -3835,13 +3873,10 @@
       <c r="C21" s="70"/>
       <c r="D21" s="70"/>
       <c r="G21" s="104"/>
-      <c r="H21" s="105" t="n">
-        <f aca="false">H20</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H21" s="105"/>
       <c r="I21" s="94" t="n">
         <f aca="false">(H21/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J21" s="106"/>
       <c r="K21" s="107"/>
@@ -3855,13 +3890,10 @@
       <c r="C22" s="70"/>
       <c r="D22" s="70"/>
       <c r="G22" s="104"/>
-      <c r="H22" s="105" t="n">
-        <f aca="false">H21</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H22" s="105"/>
       <c r="I22" s="94" t="n">
         <f aca="false">(H22/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J22" s="106"/>
       <c r="K22" s="107"/>
@@ -3875,13 +3907,10 @@
       <c r="C23" s="70"/>
       <c r="D23" s="70"/>
       <c r="G23" s="104"/>
-      <c r="H23" s="105" t="n">
-        <f aca="false">H22</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H23" s="105"/>
       <c r="I23" s="94" t="n">
         <f aca="false">(H23/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J23" s="106"/>
       <c r="K23" s="107"/>
@@ -3895,13 +3924,10 @@
       <c r="C24" s="70"/>
       <c r="D24" s="70"/>
       <c r="G24" s="104"/>
-      <c r="H24" s="105" t="n">
-        <f aca="false">H23</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H24" s="105"/>
       <c r="I24" s="94" t="n">
         <f aca="false">(H24/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J24" s="106"/>
       <c r="K24" s="107"/>
@@ -3915,13 +3941,10 @@
       <c r="C25" s="70"/>
       <c r="D25" s="70"/>
       <c r="G25" s="104"/>
-      <c r="H25" s="105" t="n">
-        <f aca="false">H24</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H25" s="105"/>
       <c r="I25" s="94" t="n">
         <f aca="false">(H25/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J25" s="106"/>
       <c r="K25" s="107"/>
@@ -3935,13 +3958,10 @@
       <c r="C26" s="70"/>
       <c r="D26" s="70"/>
       <c r="G26" s="104"/>
-      <c r="H26" s="105" t="n">
-        <f aca="false">H25</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H26" s="105"/>
       <c r="I26" s="94" t="n">
         <f aca="false">(H26/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J26" s="106"/>
       <c r="K26" s="107"/>
@@ -3955,13 +3975,10 @@
       <c r="C27" s="70"/>
       <c r="D27" s="70"/>
       <c r="G27" s="104"/>
-      <c r="H27" s="105" t="n">
-        <f aca="false">H26</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H27" s="105"/>
       <c r="I27" s="94" t="n">
         <f aca="false">(H27/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J27" s="106"/>
       <c r="K27" s="107"/>
@@ -3975,13 +3992,10 @@
       <c r="C28" s="70"/>
       <c r="D28" s="70"/>
       <c r="G28" s="104"/>
-      <c r="H28" s="105" t="n">
-        <f aca="false">H27</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H28" s="105"/>
       <c r="I28" s="94" t="n">
         <f aca="false">(H28/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J28" s="106"/>
       <c r="K28" s="107"/>
@@ -3995,13 +4009,10 @@
       <c r="C29" s="70"/>
       <c r="D29" s="70"/>
       <c r="G29" s="104"/>
-      <c r="H29" s="105" t="n">
-        <f aca="false">H28</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H29" s="105"/>
       <c r="I29" s="94" t="n">
         <f aca="false">(H29/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J29" s="106"/>
       <c r="K29" s="107"/>
@@ -4015,13 +4026,10 @@
       <c r="C30" s="70"/>
       <c r="D30" s="70"/>
       <c r="G30" s="104"/>
-      <c r="H30" s="105" t="n">
-        <f aca="false">H29</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H30" s="105"/>
       <c r="I30" s="94" t="n">
         <f aca="false">(H30/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J30" s="106"/>
       <c r="K30" s="107"/>
@@ -4035,13 +4043,10 @@
       <c r="C31" s="70"/>
       <c r="D31" s="70"/>
       <c r="G31" s="104"/>
-      <c r="H31" s="105" t="n">
-        <f aca="false">H30</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H31" s="105"/>
       <c r="I31" s="94" t="n">
         <f aca="false">(H31/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J31" s="106"/>
       <c r="K31" s="107"/>
@@ -4055,13 +4060,10 @@
       <c r="C32" s="70"/>
       <c r="D32" s="70"/>
       <c r="G32" s="104"/>
-      <c r="H32" s="105" t="n">
-        <f aca="false">H31</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H32" s="105"/>
       <c r="I32" s="94" t="n">
         <f aca="false">(H32/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J32" s="106"/>
       <c r="K32" s="107"/>
@@ -4075,13 +4077,10 @@
       <c r="C33" s="70"/>
       <c r="D33" s="70"/>
       <c r="G33" s="104"/>
-      <c r="H33" s="105" t="n">
-        <f aca="false">H32</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H33" s="105"/>
       <c r="I33" s="94" t="n">
         <f aca="false">(H33/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J33" s="106"/>
       <c r="K33" s="107"/>
@@ -4095,13 +4094,10 @@
       <c r="C34" s="70"/>
       <c r="D34" s="70"/>
       <c r="G34" s="104"/>
-      <c r="H34" s="105" t="n">
-        <f aca="false">H33</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H34" s="105"/>
       <c r="I34" s="94" t="n">
         <f aca="false">(H34/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J34" s="106"/>
       <c r="K34" s="107"/>
@@ -4111,17 +4107,14 @@
       <c r="O34" s="111"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="112"/>
-      <c r="C35" s="112"/>
-      <c r="D35" s="112"/>
+      <c r="B35" s="115"/>
+      <c r="C35" s="115"/>
+      <c r="D35" s="115"/>
       <c r="G35" s="104"/>
-      <c r="H35" s="105" t="n">
-        <f aca="false">H34</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H35" s="105"/>
       <c r="I35" s="94" t="n">
         <f aca="false">(H35/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J35" s="106"/>
       <c r="K35" s="107"/>
@@ -4131,17 +4124,14 @@
       <c r="O35" s="111"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="112"/>
-      <c r="C36" s="112"/>
-      <c r="D36" s="112"/>
+      <c r="B36" s="115"/>
+      <c r="C36" s="115"/>
+      <c r="D36" s="115"/>
       <c r="G36" s="104"/>
-      <c r="H36" s="105" t="n">
-        <f aca="false">H35</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H36" s="105"/>
       <c r="I36" s="94" t="n">
         <f aca="false">(H36/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J36" s="106"/>
       <c r="K36" s="107"/>
@@ -4152,13 +4142,10 @@
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G37" s="104"/>
-      <c r="H37" s="105" t="n">
-        <f aca="false">H36</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H37" s="105"/>
       <c r="I37" s="94" t="n">
         <f aca="false">(H37/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J37" s="106"/>
       <c r="K37" s="107"/>
@@ -4169,13 +4156,10 @@
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G38" s="104"/>
-      <c r="H38" s="105" t="n">
-        <f aca="false">H37</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H38" s="105"/>
       <c r="I38" s="94" t="n">
         <f aca="false">(H38/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J38" s="106"/>
       <c r="K38" s="107"/>
@@ -4186,13 +4170,10 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G39" s="104"/>
-      <c r="H39" s="105" t="n">
-        <f aca="false">H38</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H39" s="105"/>
       <c r="I39" s="94" t="n">
         <f aca="false">(H39/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J39" s="106"/>
       <c r="K39" s="107"/>
@@ -4203,13 +4184,10 @@
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G40" s="104"/>
-      <c r="H40" s="105" t="n">
-        <f aca="false">H39</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H40" s="105"/>
       <c r="I40" s="94" t="n">
         <f aca="false">(H40/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J40" s="106"/>
       <c r="K40" s="107"/>
@@ -4220,13 +4198,10 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G41" s="104"/>
-      <c r="H41" s="105" t="n">
-        <f aca="false">H40</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H41" s="105"/>
       <c r="I41" s="94" t="n">
         <f aca="false">(H41/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J41" s="106"/>
       <c r="K41" s="107"/>
@@ -4237,13 +4212,10 @@
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G42" s="104"/>
-      <c r="H42" s="105" t="n">
-        <f aca="false">H41</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H42" s="105"/>
       <c r="I42" s="94" t="n">
         <f aca="false">(H42/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J42" s="106"/>
       <c r="K42" s="107"/>
@@ -4254,13 +4226,10 @@
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G43" s="104"/>
-      <c r="H43" s="105" t="n">
-        <f aca="false">H42</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H43" s="105"/>
       <c r="I43" s="94" t="n">
         <f aca="false">(H43/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J43" s="106"/>
       <c r="K43" s="107"/>
@@ -4271,13 +4240,10 @@
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G44" s="104"/>
-      <c r="H44" s="105" t="n">
-        <f aca="false">H43</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="H44" s="105"/>
       <c r="I44" s="94" t="n">
         <f aca="false">(H44/C2)/10</f>
-        <v>27.5510204081633</v>
+        <v>0</v>
       </c>
       <c r="J44" s="106"/>
       <c r="K44" s="107"/>
@@ -4287,21 +4253,18 @@
       <c r="O44" s="111"/>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G45" s="113"/>
-      <c r="H45" s="105" t="n">
-        <f aca="false">H44</f>
-        <v>474.428571428571</v>
-      </c>
+      <c r="G45" s="116"/>
+      <c r="H45" s="105"/>
       <c r="I45" s="94" t="n">
         <f aca="false">(H45/C2)/10</f>
-        <v>27.5510204081633</v>
-      </c>
-      <c r="J45" s="114"/>
-      <c r="K45" s="115"/>
-      <c r="L45" s="116"/>
-      <c r="M45" s="117"/>
-      <c r="N45" s="118"/>
-      <c r="O45" s="119"/>
+        <v>0</v>
+      </c>
+      <c r="J45" s="117"/>
+      <c r="K45" s="118"/>
+      <c r="L45" s="119"/>
+      <c r="M45" s="120"/>
+      <c r="N45" s="121"/>
+      <c r="O45" s="122"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -4357,7 +4320,7 @@
         <v>106</v>
       </c>
       <c r="D1" s="74" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E1" s="74" t="s">
         <v>108</v>
@@ -4552,12 +4515,12 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="101"/>
-      <c r="B17" s="102"/>
-      <c r="C17" s="102"/>
-      <c r="D17" s="102"/>
-      <c r="E17" s="103"/>
-      <c r="F17" s="103"/>
+      <c r="A17" s="102"/>
+      <c r="B17" s="103"/>
+      <c r="C17" s="103"/>
+      <c r="D17" s="103"/>
+      <c r="E17" s="101"/>
+      <c r="F17" s="101"/>
       <c r="G17" s="92"/>
       <c r="H17" s="105" t="n">
         <f aca="false">E2</f>
@@ -4915,9 +4878,9 @@
       <c r="O34" s="111"/>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="112"/>
-      <c r="C35" s="112"/>
-      <c r="D35" s="112"/>
+      <c r="B35" s="115"/>
+      <c r="C35" s="115"/>
+      <c r="D35" s="115"/>
       <c r="G35" s="104"/>
       <c r="H35" s="105" t="n">
         <f aca="false">H34</f>
@@ -4935,9 +4898,9 @@
       <c r="O35" s="111"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="112"/>
-      <c r="C36" s="112"/>
-      <c r="D36" s="112"/>
+      <c r="B36" s="115"/>
+      <c r="C36" s="115"/>
+      <c r="D36" s="115"/>
       <c r="G36" s="104"/>
       <c r="H36" s="105" t="n">
         <f aca="false">H35</f>
@@ -5091,7 +5054,7 @@
       <c r="O44" s="111"/>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G45" s="113"/>
+      <c r="G45" s="116"/>
       <c r="H45" s="105" t="n">
         <f aca="false">H44</f>
         <v>362</v>
@@ -5100,12 +5063,12 @@
         <f aca="false">(H45/C2)/10</f>
         <v>51.7142857142857</v>
       </c>
-      <c r="J45" s="114"/>
-      <c r="K45" s="115"/>
-      <c r="L45" s="116"/>
-      <c r="M45" s="117"/>
-      <c r="N45" s="118"/>
-      <c r="O45" s="119"/>
+      <c r="J45" s="117"/>
+      <c r="K45" s="118"/>
+      <c r="L45" s="119"/>
+      <c r="M45" s="120"/>
+      <c r="N45" s="121"/>
+      <c r="O45" s="122"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -5134,6 +5097,655 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:L44"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="22" width="15.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="22" width="16.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="22" width="20.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="22" width="21.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="22" width="16.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="22" width="20.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="70" width="15.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="71" width="14.92"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="9" min="9" style="71" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="10" min="10" style="72" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="12" min="11" style="71" width="11.53"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="73"/>
+      <c r="B1" s="74" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="74" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" s="74" t="s">
+        <v>121</v>
+      </c>
+      <c r="E1" s="74" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" s="74" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="67" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="76" t="n">
+        <f aca="false">(E2/C2)/10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="68" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" s="71"/>
+      <c r="C3" s="71" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="D3" s="75"/>
+      <c r="E3" s="75"/>
+      <c r="F3" s="76" t="n">
+        <f aca="false">(E3/C3)/10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="73"/>
+      <c r="B7" s="73" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" s="73" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="73" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" s="73" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="73"/>
+      <c r="E8" s="1" t="e">
+        <f aca="false">E2/D2</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="73"/>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G12" s="77" t="s">
+        <v>122</v>
+      </c>
+      <c r="H12" s="77"/>
+      <c r="I12" s="77"/>
+      <c r="J12" s="78" t="s">
+        <v>123</v>
+      </c>
+      <c r="K12" s="78"/>
+      <c r="L12" s="78"/>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G13" s="80" t="s">
+        <v>116</v>
+      </c>
+      <c r="H13" s="81" t="s">
+        <v>117</v>
+      </c>
+      <c r="I13" s="81"/>
+      <c r="J13" s="82" t="s">
+        <v>116</v>
+      </c>
+      <c r="K13" s="83" t="s">
+        <v>117</v>
+      </c>
+      <c r="L13" s="83"/>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G14" s="80"/>
+      <c r="H14" s="86" t="s">
+        <v>118</v>
+      </c>
+      <c r="I14" s="87" t="s">
+        <v>119</v>
+      </c>
+      <c r="J14" s="82"/>
+      <c r="K14" s="88" t="s">
+        <v>118</v>
+      </c>
+      <c r="L14" s="89" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="73"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="G15" s="92" t="n">
+        <v>46202</v>
+      </c>
+      <c r="H15" s="94" t="n">
+        <f aca="false">E2</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="94" t="n">
+        <f aca="false">F2</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="95"/>
+      <c r="K15" s="96"/>
+      <c r="L15" s="97" t="n">
+        <f aca="false">(K15/C3)/10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="102"/>
+      <c r="B16" s="103"/>
+      <c r="C16" s="103"/>
+      <c r="D16" s="103"/>
+      <c r="E16" s="101"/>
+      <c r="F16" s="101"/>
+      <c r="G16" s="92"/>
+      <c r="H16" s="105" t="n">
+        <f aca="false">E2</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="94" t="n">
+        <f aca="false">(H16/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="106"/>
+      <c r="K16" s="107"/>
+      <c r="L16" s="108"/>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="70"/>
+      <c r="C17" s="70"/>
+      <c r="D17" s="70"/>
+      <c r="G17" s="104"/>
+      <c r="H17" s="105" t="n">
+        <f aca="false">H16</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="94" t="n">
+        <f aca="false">(H17/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="106"/>
+      <c r="K17" s="107"/>
+      <c r="L17" s="108"/>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="70"/>
+      <c r="C18" s="70"/>
+      <c r="D18" s="70"/>
+      <c r="G18" s="104"/>
+      <c r="H18" s="105" t="n">
+        <f aca="false">H17</f>
+        <v>0</v>
+      </c>
+      <c r="I18" s="94" t="n">
+        <f aca="false">(H18/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="106"/>
+      <c r="K18" s="107"/>
+      <c r="L18" s="108"/>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="70"/>
+      <c r="C19" s="70"/>
+      <c r="D19" s="70"/>
+      <c r="G19" s="104"/>
+      <c r="H19" s="105" t="n">
+        <f aca="false">H18</f>
+        <v>0</v>
+      </c>
+      <c r="I19" s="94" t="n">
+        <f aca="false">(H19/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="106"/>
+      <c r="K19" s="107"/>
+      <c r="L19" s="108"/>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="70"/>
+      <c r="C20" s="70"/>
+      <c r="D20" s="70"/>
+      <c r="G20" s="104"/>
+      <c r="H20" s="105" t="n">
+        <f aca="false">H19</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="94" t="n">
+        <f aca="false">(H20/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="106"/>
+      <c r="K20" s="107"/>
+      <c r="L20" s="108"/>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="70"/>
+      <c r="C21" s="70"/>
+      <c r="D21" s="70"/>
+      <c r="G21" s="104"/>
+      <c r="H21" s="105" t="n">
+        <f aca="false">H20</f>
+        <v>0</v>
+      </c>
+      <c r="I21" s="94" t="n">
+        <f aca="false">(H21/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="106"/>
+      <c r="K21" s="107"/>
+      <c r="L21" s="108"/>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="70"/>
+      <c r="C22" s="70"/>
+      <c r="D22" s="70"/>
+      <c r="G22" s="104"/>
+      <c r="H22" s="105" t="n">
+        <f aca="false">H21</f>
+        <v>0</v>
+      </c>
+      <c r="I22" s="94" t="n">
+        <f aca="false">(H22/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="106"/>
+      <c r="K22" s="107"/>
+      <c r="L22" s="108"/>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="70"/>
+      <c r="C23" s="70"/>
+      <c r="D23" s="70"/>
+      <c r="G23" s="104"/>
+      <c r="H23" s="105" t="n">
+        <f aca="false">H22</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="94" t="n">
+        <f aca="false">(H23/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="106"/>
+      <c r="K23" s="107"/>
+      <c r="L23" s="108"/>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="70"/>
+      <c r="C24" s="70"/>
+      <c r="D24" s="70"/>
+      <c r="G24" s="104"/>
+      <c r="H24" s="105" t="n">
+        <f aca="false">H23</f>
+        <v>0</v>
+      </c>
+      <c r="I24" s="94" t="n">
+        <f aca="false">(H24/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="106"/>
+      <c r="K24" s="107"/>
+      <c r="L24" s="108"/>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="70"/>
+      <c r="C25" s="70"/>
+      <c r="D25" s="70"/>
+      <c r="G25" s="104"/>
+      <c r="H25" s="105" t="n">
+        <f aca="false">H24</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="94" t="n">
+        <f aca="false">(H25/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J25" s="106"/>
+      <c r="K25" s="107"/>
+      <c r="L25" s="108"/>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="70"/>
+      <c r="C26" s="70"/>
+      <c r="D26" s="70"/>
+      <c r="G26" s="104"/>
+      <c r="H26" s="105" t="n">
+        <f aca="false">H25</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="94" t="n">
+        <f aca="false">(H26/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J26" s="106"/>
+      <c r="K26" s="107"/>
+      <c r="L26" s="108"/>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="70"/>
+      <c r="C27" s="70"/>
+      <c r="D27" s="70"/>
+      <c r="G27" s="104"/>
+      <c r="H27" s="105" t="n">
+        <f aca="false">H26</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="94" t="n">
+        <f aca="false">(H27/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="106"/>
+      <c r="K27" s="107"/>
+      <c r="L27" s="108"/>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="70"/>
+      <c r="C28" s="70"/>
+      <c r="D28" s="70"/>
+      <c r="G28" s="104"/>
+      <c r="H28" s="105" t="n">
+        <f aca="false">H27</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="94" t="n">
+        <f aca="false">(H28/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J28" s="106"/>
+      <c r="K28" s="107"/>
+      <c r="L28" s="108"/>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="70"/>
+      <c r="C29" s="70"/>
+      <c r="D29" s="70"/>
+      <c r="G29" s="104"/>
+      <c r="H29" s="105" t="n">
+        <f aca="false">H28</f>
+        <v>0</v>
+      </c>
+      <c r="I29" s="94" t="n">
+        <f aca="false">(H29/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J29" s="106"/>
+      <c r="K29" s="107"/>
+      <c r="L29" s="108"/>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="70"/>
+      <c r="C30" s="70"/>
+      <c r="D30" s="70"/>
+      <c r="G30" s="104"/>
+      <c r="H30" s="105" t="n">
+        <f aca="false">H29</f>
+        <v>0</v>
+      </c>
+      <c r="I30" s="94" t="n">
+        <f aca="false">(H30/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="106"/>
+      <c r="K30" s="107"/>
+      <c r="L30" s="108"/>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="70"/>
+      <c r="C31" s="70"/>
+      <c r="D31" s="70"/>
+      <c r="G31" s="104"/>
+      <c r="H31" s="105" t="n">
+        <f aca="false">H30</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="94" t="n">
+        <f aca="false">(H31/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="106"/>
+      <c r="K31" s="107"/>
+      <c r="L31" s="108"/>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="70"/>
+      <c r="C32" s="70"/>
+      <c r="D32" s="70"/>
+      <c r="G32" s="104"/>
+      <c r="H32" s="105" t="n">
+        <f aca="false">H31</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="94" t="n">
+        <f aca="false">(H32/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="106"/>
+      <c r="K32" s="107"/>
+      <c r="L32" s="108"/>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="70"/>
+      <c r="C33" s="70"/>
+      <c r="D33" s="70"/>
+      <c r="G33" s="104"/>
+      <c r="H33" s="105" t="n">
+        <f aca="false">H32</f>
+        <v>0</v>
+      </c>
+      <c r="I33" s="94" t="n">
+        <f aca="false">(H33/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J33" s="106"/>
+      <c r="K33" s="107"/>
+      <c r="L33" s="108"/>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="115"/>
+      <c r="C34" s="115"/>
+      <c r="D34" s="115"/>
+      <c r="G34" s="104"/>
+      <c r="H34" s="105" t="n">
+        <f aca="false">H33</f>
+        <v>0</v>
+      </c>
+      <c r="I34" s="94" t="n">
+        <f aca="false">(H34/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J34" s="106"/>
+      <c r="K34" s="107"/>
+      <c r="L34" s="108"/>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="115"/>
+      <c r="C35" s="115"/>
+      <c r="D35" s="115"/>
+      <c r="G35" s="104"/>
+      <c r="H35" s="105" t="n">
+        <f aca="false">H34</f>
+        <v>0</v>
+      </c>
+      <c r="I35" s="94" t="n">
+        <f aca="false">(H35/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J35" s="106"/>
+      <c r="K35" s="107"/>
+      <c r="L35" s="108"/>
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G36" s="104"/>
+      <c r="H36" s="105" t="n">
+        <f aca="false">H35</f>
+        <v>0</v>
+      </c>
+      <c r="I36" s="94" t="n">
+        <f aca="false">(H36/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J36" s="106"/>
+      <c r="K36" s="107"/>
+      <c r="L36" s="108"/>
+    </row>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G37" s="104"/>
+      <c r="H37" s="105" t="n">
+        <f aca="false">H36</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="94" t="n">
+        <f aca="false">(H37/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J37" s="106"/>
+      <c r="K37" s="107"/>
+      <c r="L37" s="108"/>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G38" s="104"/>
+      <c r="H38" s="105" t="n">
+        <f aca="false">H37</f>
+        <v>0</v>
+      </c>
+      <c r="I38" s="94" t="n">
+        <f aca="false">(H38/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J38" s="106"/>
+      <c r="K38" s="107"/>
+      <c r="L38" s="108"/>
+    </row>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G39" s="104"/>
+      <c r="H39" s="105" t="n">
+        <f aca="false">H38</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="94" t="n">
+        <f aca="false">(H39/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J39" s="106"/>
+      <c r="K39" s="107"/>
+      <c r="L39" s="108"/>
+    </row>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G40" s="104"/>
+      <c r="H40" s="105" t="n">
+        <f aca="false">H39</f>
+        <v>0</v>
+      </c>
+      <c r="I40" s="94" t="n">
+        <f aca="false">(H40/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J40" s="106"/>
+      <c r="K40" s="107"/>
+      <c r="L40" s="108"/>
+    </row>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G41" s="104"/>
+      <c r="H41" s="105" t="n">
+        <f aca="false">H40</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="94" t="n">
+        <f aca="false">(H41/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J41" s="106"/>
+      <c r="K41" s="107"/>
+      <c r="L41" s="108"/>
+    </row>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G42" s="104"/>
+      <c r="H42" s="105" t="n">
+        <f aca="false">H41</f>
+        <v>0</v>
+      </c>
+      <c r="I42" s="94" t="n">
+        <f aca="false">(H42/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J42" s="106"/>
+      <c r="K42" s="107"/>
+      <c r="L42" s="108"/>
+    </row>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G43" s="104"/>
+      <c r="H43" s="105" t="n">
+        <f aca="false">H42</f>
+        <v>0</v>
+      </c>
+      <c r="I43" s="94" t="n">
+        <f aca="false">(H43/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J43" s="106"/>
+      <c r="K43" s="107"/>
+      <c r="L43" s="108"/>
+    </row>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G44" s="116"/>
+      <c r="H44" s="105" t="n">
+        <f aca="false">H43</f>
+        <v>0</v>
+      </c>
+      <c r="I44" s="94" t="n">
+        <f aca="false">(H44/C2)/10</f>
+        <v>0</v>
+      </c>
+      <c r="J44" s="117"/>
+      <c r="K44" s="118"/>
+      <c r="L44" s="119"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="J13:J14"/>
+    <mergeCell ref="K13:L13"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="B1:J34"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
@@ -5202,334 +5814,334 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="120"/>
-      <c r="C5" s="121"/>
-      <c r="D5" s="121"/>
-      <c r="E5" s="122"/>
-      <c r="F5" s="123"/>
-      <c r="G5" s="123"/>
-      <c r="H5" s="124"/>
-      <c r="I5" s="125"/>
-      <c r="J5" s="126"/>
+      <c r="B5" s="123"/>
+      <c r="C5" s="124"/>
+      <c r="D5" s="124"/>
+      <c r="E5" s="125"/>
+      <c r="F5" s="126"/>
+      <c r="G5" s="126"/>
+      <c r="H5" s="127"/>
+      <c r="I5" s="128"/>
+      <c r="J5" s="129"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="127"/>
-      <c r="C6" s="128"/>
-      <c r="D6" s="128"/>
-      <c r="E6" s="129"/>
-      <c r="F6" s="130"/>
-      <c r="G6" s="130"/>
-      <c r="H6" s="131"/>
-      <c r="I6" s="132"/>
-      <c r="J6" s="133"/>
+      <c r="B6" s="130"/>
+      <c r="C6" s="131"/>
+      <c r="D6" s="131"/>
+      <c r="E6" s="132"/>
+      <c r="F6" s="133"/>
+      <c r="G6" s="133"/>
+      <c r="H6" s="134"/>
+      <c r="I6" s="135"/>
+      <c r="J6" s="136"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="127"/>
-      <c r="C7" s="128"/>
-      <c r="D7" s="128"/>
-      <c r="E7" s="129"/>
-      <c r="F7" s="130"/>
-      <c r="G7" s="130"/>
-      <c r="H7" s="131"/>
-      <c r="I7" s="132"/>
-      <c r="J7" s="133"/>
+      <c r="B7" s="130"/>
+      <c r="C7" s="131"/>
+      <c r="D7" s="131"/>
+      <c r="E7" s="132"/>
+      <c r="F7" s="133"/>
+      <c r="G7" s="133"/>
+      <c r="H7" s="134"/>
+      <c r="I7" s="135"/>
+      <c r="J7" s="136"/>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="127"/>
-      <c r="C8" s="128"/>
-      <c r="D8" s="128"/>
-      <c r="E8" s="129"/>
-      <c r="F8" s="130"/>
-      <c r="G8" s="130"/>
-      <c r="H8" s="131"/>
-      <c r="I8" s="132"/>
-      <c r="J8" s="133"/>
+      <c r="B8" s="130"/>
+      <c r="C8" s="131"/>
+      <c r="D8" s="131"/>
+      <c r="E8" s="132"/>
+      <c r="F8" s="133"/>
+      <c r="G8" s="133"/>
+      <c r="H8" s="134"/>
+      <c r="I8" s="135"/>
+      <c r="J8" s="136"/>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="127"/>
-      <c r="C9" s="128"/>
-      <c r="D9" s="128"/>
-      <c r="E9" s="129"/>
-      <c r="F9" s="130"/>
-      <c r="G9" s="130"/>
-      <c r="H9" s="131"/>
-      <c r="I9" s="132"/>
-      <c r="J9" s="133"/>
+      <c r="B9" s="130"/>
+      <c r="C9" s="131"/>
+      <c r="D9" s="131"/>
+      <c r="E9" s="132"/>
+      <c r="F9" s="133"/>
+      <c r="G9" s="133"/>
+      <c r="H9" s="134"/>
+      <c r="I9" s="135"/>
+      <c r="J9" s="136"/>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="127"/>
-      <c r="C10" s="128"/>
-      <c r="D10" s="128"/>
-      <c r="E10" s="129"/>
-      <c r="F10" s="130"/>
-      <c r="G10" s="130"/>
-      <c r="H10" s="131"/>
-      <c r="I10" s="132"/>
-      <c r="J10" s="133"/>
+      <c r="B10" s="130"/>
+      <c r="C10" s="131"/>
+      <c r="D10" s="131"/>
+      <c r="E10" s="132"/>
+      <c r="F10" s="133"/>
+      <c r="G10" s="133"/>
+      <c r="H10" s="134"/>
+      <c r="I10" s="135"/>
+      <c r="J10" s="136"/>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="127"/>
-      <c r="C11" s="128"/>
-      <c r="D11" s="128"/>
-      <c r="E11" s="129"/>
-      <c r="F11" s="130"/>
-      <c r="G11" s="130"/>
-      <c r="H11" s="131"/>
-      <c r="I11" s="132"/>
-      <c r="J11" s="133"/>
+      <c r="B11" s="130"/>
+      <c r="C11" s="131"/>
+      <c r="D11" s="131"/>
+      <c r="E11" s="132"/>
+      <c r="F11" s="133"/>
+      <c r="G11" s="133"/>
+      <c r="H11" s="134"/>
+      <c r="I11" s="135"/>
+      <c r="J11" s="136"/>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="127"/>
-      <c r="C12" s="128"/>
-      <c r="D12" s="128"/>
-      <c r="E12" s="129"/>
-      <c r="F12" s="130"/>
-      <c r="G12" s="130"/>
-      <c r="H12" s="131"/>
-      <c r="I12" s="132"/>
-      <c r="J12" s="133"/>
+      <c r="B12" s="130"/>
+      <c r="C12" s="131"/>
+      <c r="D12" s="131"/>
+      <c r="E12" s="132"/>
+      <c r="F12" s="133"/>
+      <c r="G12" s="133"/>
+      <c r="H12" s="134"/>
+      <c r="I12" s="135"/>
+      <c r="J12" s="136"/>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="127"/>
-      <c r="C13" s="128"/>
-      <c r="D13" s="128"/>
-      <c r="E13" s="129"/>
-      <c r="F13" s="130"/>
-      <c r="G13" s="130"/>
-      <c r="H13" s="131"/>
-      <c r="I13" s="132"/>
-      <c r="J13" s="133"/>
+      <c r="B13" s="130"/>
+      <c r="C13" s="131"/>
+      <c r="D13" s="131"/>
+      <c r="E13" s="132"/>
+      <c r="F13" s="133"/>
+      <c r="G13" s="133"/>
+      <c r="H13" s="134"/>
+      <c r="I13" s="135"/>
+      <c r="J13" s="136"/>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="127"/>
-      <c r="C14" s="128"/>
-      <c r="D14" s="128"/>
-      <c r="E14" s="129"/>
-      <c r="F14" s="130"/>
-      <c r="G14" s="130"/>
-      <c r="H14" s="131"/>
-      <c r="I14" s="132"/>
-      <c r="J14" s="133"/>
+      <c r="B14" s="130"/>
+      <c r="C14" s="131"/>
+      <c r="D14" s="131"/>
+      <c r="E14" s="132"/>
+      <c r="F14" s="133"/>
+      <c r="G14" s="133"/>
+      <c r="H14" s="134"/>
+      <c r="I14" s="135"/>
+      <c r="J14" s="136"/>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="127"/>
-      <c r="C15" s="128"/>
-      <c r="D15" s="128"/>
-      <c r="E15" s="129"/>
-      <c r="F15" s="130"/>
-      <c r="G15" s="130"/>
-      <c r="H15" s="131"/>
-      <c r="I15" s="132"/>
-      <c r="J15" s="133"/>
+      <c r="B15" s="130"/>
+      <c r="C15" s="131"/>
+      <c r="D15" s="131"/>
+      <c r="E15" s="132"/>
+      <c r="F15" s="133"/>
+      <c r="G15" s="133"/>
+      <c r="H15" s="134"/>
+      <c r="I15" s="135"/>
+      <c r="J15" s="136"/>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="127"/>
-      <c r="C16" s="128"/>
-      <c r="D16" s="128"/>
-      <c r="E16" s="129"/>
-      <c r="F16" s="130"/>
-      <c r="G16" s="130"/>
-      <c r="H16" s="131"/>
-      <c r="I16" s="132"/>
-      <c r="J16" s="133"/>
+      <c r="B16" s="130"/>
+      <c r="C16" s="131"/>
+      <c r="D16" s="131"/>
+      <c r="E16" s="132"/>
+      <c r="F16" s="133"/>
+      <c r="G16" s="133"/>
+      <c r="H16" s="134"/>
+      <c r="I16" s="135"/>
+      <c r="J16" s="136"/>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="127"/>
-      <c r="C17" s="128"/>
-      <c r="D17" s="128"/>
-      <c r="E17" s="129"/>
-      <c r="F17" s="130"/>
-      <c r="G17" s="130"/>
-      <c r="H17" s="131"/>
-      <c r="I17" s="132"/>
-      <c r="J17" s="133"/>
+      <c r="B17" s="130"/>
+      <c r="C17" s="131"/>
+      <c r="D17" s="131"/>
+      <c r="E17" s="132"/>
+      <c r="F17" s="133"/>
+      <c r="G17" s="133"/>
+      <c r="H17" s="134"/>
+      <c r="I17" s="135"/>
+      <c r="J17" s="136"/>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="127"/>
-      <c r="C18" s="128"/>
-      <c r="D18" s="128"/>
-      <c r="E18" s="129"/>
-      <c r="F18" s="130"/>
-      <c r="G18" s="130"/>
-      <c r="H18" s="131"/>
-      <c r="I18" s="132"/>
-      <c r="J18" s="133"/>
+      <c r="B18" s="130"/>
+      <c r="C18" s="131"/>
+      <c r="D18" s="131"/>
+      <c r="E18" s="132"/>
+      <c r="F18" s="133"/>
+      <c r="G18" s="133"/>
+      <c r="H18" s="134"/>
+      <c r="I18" s="135"/>
+      <c r="J18" s="136"/>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="127"/>
-      <c r="C19" s="128"/>
-      <c r="D19" s="128"/>
-      <c r="E19" s="129"/>
-      <c r="F19" s="130"/>
-      <c r="G19" s="130"/>
-      <c r="H19" s="131"/>
-      <c r="I19" s="132"/>
-      <c r="J19" s="133"/>
+      <c r="B19" s="130"/>
+      <c r="C19" s="131"/>
+      <c r="D19" s="131"/>
+      <c r="E19" s="132"/>
+      <c r="F19" s="133"/>
+      <c r="G19" s="133"/>
+      <c r="H19" s="134"/>
+      <c r="I19" s="135"/>
+      <c r="J19" s="136"/>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="127"/>
-      <c r="C20" s="128"/>
-      <c r="D20" s="128"/>
-      <c r="E20" s="129"/>
-      <c r="F20" s="130"/>
-      <c r="G20" s="130"/>
-      <c r="H20" s="131"/>
-      <c r="I20" s="132"/>
-      <c r="J20" s="133"/>
+      <c r="B20" s="130"/>
+      <c r="C20" s="131"/>
+      <c r="D20" s="131"/>
+      <c r="E20" s="132"/>
+      <c r="F20" s="133"/>
+      <c r="G20" s="133"/>
+      <c r="H20" s="134"/>
+      <c r="I20" s="135"/>
+      <c r="J20" s="136"/>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="127"/>
-      <c r="C21" s="128"/>
-      <c r="D21" s="128"/>
-      <c r="E21" s="129"/>
-      <c r="F21" s="130"/>
-      <c r="G21" s="130"/>
-      <c r="H21" s="131"/>
-      <c r="I21" s="132"/>
-      <c r="J21" s="133"/>
+      <c r="B21" s="130"/>
+      <c r="C21" s="131"/>
+      <c r="D21" s="131"/>
+      <c r="E21" s="132"/>
+      <c r="F21" s="133"/>
+      <c r="G21" s="133"/>
+      <c r="H21" s="134"/>
+      <c r="I21" s="135"/>
+      <c r="J21" s="136"/>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="127"/>
-      <c r="C22" s="128"/>
-      <c r="D22" s="128"/>
-      <c r="E22" s="129"/>
-      <c r="F22" s="130"/>
-      <c r="G22" s="130"/>
-      <c r="H22" s="131"/>
-      <c r="I22" s="132"/>
-      <c r="J22" s="133"/>
+      <c r="B22" s="130"/>
+      <c r="C22" s="131"/>
+      <c r="D22" s="131"/>
+      <c r="E22" s="132"/>
+      <c r="F22" s="133"/>
+      <c r="G22" s="133"/>
+      <c r="H22" s="134"/>
+      <c r="I22" s="135"/>
+      <c r="J22" s="136"/>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="127"/>
-      <c r="C23" s="128"/>
-      <c r="D23" s="128"/>
-      <c r="E23" s="129"/>
-      <c r="F23" s="130"/>
-      <c r="G23" s="130"/>
-      <c r="H23" s="131"/>
-      <c r="I23" s="132"/>
-      <c r="J23" s="133"/>
+      <c r="B23" s="130"/>
+      <c r="C23" s="131"/>
+      <c r="D23" s="131"/>
+      <c r="E23" s="132"/>
+      <c r="F23" s="133"/>
+      <c r="G23" s="133"/>
+      <c r="H23" s="134"/>
+      <c r="I23" s="135"/>
+      <c r="J23" s="136"/>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="127"/>
-      <c r="C24" s="128"/>
-      <c r="D24" s="128"/>
-      <c r="E24" s="129"/>
-      <c r="F24" s="130"/>
-      <c r="G24" s="130"/>
-      <c r="H24" s="131"/>
-      <c r="I24" s="132"/>
-      <c r="J24" s="133"/>
+      <c r="B24" s="130"/>
+      <c r="C24" s="131"/>
+      <c r="D24" s="131"/>
+      <c r="E24" s="132"/>
+      <c r="F24" s="133"/>
+      <c r="G24" s="133"/>
+      <c r="H24" s="134"/>
+      <c r="I24" s="135"/>
+      <c r="J24" s="136"/>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="127"/>
-      <c r="C25" s="128"/>
-      <c r="D25" s="128"/>
-      <c r="E25" s="129"/>
-      <c r="F25" s="130"/>
-      <c r="G25" s="130"/>
-      <c r="H25" s="131"/>
-      <c r="I25" s="132"/>
-      <c r="J25" s="133"/>
+      <c r="B25" s="130"/>
+      <c r="C25" s="131"/>
+      <c r="D25" s="131"/>
+      <c r="E25" s="132"/>
+      <c r="F25" s="133"/>
+      <c r="G25" s="133"/>
+      <c r="H25" s="134"/>
+      <c r="I25" s="135"/>
+      <c r="J25" s="136"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="127"/>
-      <c r="C26" s="128"/>
-      <c r="D26" s="128"/>
-      <c r="E26" s="129"/>
-      <c r="F26" s="130"/>
-      <c r="G26" s="130"/>
-      <c r="H26" s="131"/>
-      <c r="I26" s="132"/>
-      <c r="J26" s="133"/>
+      <c r="B26" s="130"/>
+      <c r="C26" s="131"/>
+      <c r="D26" s="131"/>
+      <c r="E26" s="132"/>
+      <c r="F26" s="133"/>
+      <c r="G26" s="133"/>
+      <c r="H26" s="134"/>
+      <c r="I26" s="135"/>
+      <c r="J26" s="136"/>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="127"/>
-      <c r="C27" s="128"/>
-      <c r="D27" s="128"/>
-      <c r="E27" s="129"/>
-      <c r="F27" s="130"/>
-      <c r="G27" s="130"/>
-      <c r="H27" s="131"/>
-      <c r="I27" s="132"/>
-      <c r="J27" s="133"/>
+      <c r="B27" s="130"/>
+      <c r="C27" s="131"/>
+      <c r="D27" s="131"/>
+      <c r="E27" s="132"/>
+      <c r="F27" s="133"/>
+      <c r="G27" s="133"/>
+      <c r="H27" s="134"/>
+      <c r="I27" s="135"/>
+      <c r="J27" s="136"/>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="127"/>
-      <c r="C28" s="128"/>
-      <c r="D28" s="128"/>
-      <c r="E28" s="129"/>
-      <c r="F28" s="130"/>
-      <c r="G28" s="130"/>
-      <c r="H28" s="131"/>
-      <c r="I28" s="132"/>
-      <c r="J28" s="133"/>
+      <c r="B28" s="130"/>
+      <c r="C28" s="131"/>
+      <c r="D28" s="131"/>
+      <c r="E28" s="132"/>
+      <c r="F28" s="133"/>
+      <c r="G28" s="133"/>
+      <c r="H28" s="134"/>
+      <c r="I28" s="135"/>
+      <c r="J28" s="136"/>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="127"/>
-      <c r="C29" s="128"/>
-      <c r="D29" s="128"/>
-      <c r="E29" s="129"/>
-      <c r="F29" s="130"/>
-      <c r="G29" s="130"/>
-      <c r="H29" s="131"/>
-      <c r="I29" s="132"/>
-      <c r="J29" s="133"/>
+      <c r="B29" s="130"/>
+      <c r="C29" s="131"/>
+      <c r="D29" s="131"/>
+      <c r="E29" s="132"/>
+      <c r="F29" s="133"/>
+      <c r="G29" s="133"/>
+      <c r="H29" s="134"/>
+      <c r="I29" s="135"/>
+      <c r="J29" s="136"/>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="127"/>
-      <c r="C30" s="128"/>
-      <c r="D30" s="128"/>
-      <c r="E30" s="129"/>
-      <c r="F30" s="130"/>
-      <c r="G30" s="130"/>
-      <c r="H30" s="131"/>
-      <c r="I30" s="132"/>
-      <c r="J30" s="133"/>
+      <c r="B30" s="130"/>
+      <c r="C30" s="131"/>
+      <c r="D30" s="131"/>
+      <c r="E30" s="132"/>
+      <c r="F30" s="133"/>
+      <c r="G30" s="133"/>
+      <c r="H30" s="134"/>
+      <c r="I30" s="135"/>
+      <c r="J30" s="136"/>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="127"/>
-      <c r="C31" s="128"/>
-      <c r="D31" s="128"/>
-      <c r="E31" s="129"/>
-      <c r="F31" s="130"/>
-      <c r="G31" s="130"/>
-      <c r="H31" s="131"/>
-      <c r="I31" s="132"/>
-      <c r="J31" s="133"/>
+      <c r="B31" s="130"/>
+      <c r="C31" s="131"/>
+      <c r="D31" s="131"/>
+      <c r="E31" s="132"/>
+      <c r="F31" s="133"/>
+      <c r="G31" s="133"/>
+      <c r="H31" s="134"/>
+      <c r="I31" s="135"/>
+      <c r="J31" s="136"/>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="127"/>
-      <c r="C32" s="128"/>
-      <c r="D32" s="128"/>
-      <c r="E32" s="129"/>
-      <c r="F32" s="130"/>
-      <c r="G32" s="130"/>
-      <c r="H32" s="131"/>
-      <c r="I32" s="132"/>
-      <c r="J32" s="133"/>
+      <c r="B32" s="130"/>
+      <c r="C32" s="131"/>
+      <c r="D32" s="131"/>
+      <c r="E32" s="132"/>
+      <c r="F32" s="133"/>
+      <c r="G32" s="133"/>
+      <c r="H32" s="134"/>
+      <c r="I32" s="135"/>
+      <c r="J32" s="136"/>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="127"/>
-      <c r="C33" s="128"/>
-      <c r="D33" s="128"/>
-      <c r="E33" s="129"/>
-      <c r="F33" s="130"/>
-      <c r="G33" s="130"/>
-      <c r="H33" s="131"/>
-      <c r="I33" s="132"/>
-      <c r="J33" s="133"/>
+      <c r="B33" s="130"/>
+      <c r="C33" s="131"/>
+      <c r="D33" s="131"/>
+      <c r="E33" s="132"/>
+      <c r="F33" s="133"/>
+      <c r="G33" s="133"/>
+      <c r="H33" s="134"/>
+      <c r="I33" s="135"/>
+      <c r="J33" s="136"/>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="134"/>
-      <c r="C34" s="135"/>
-      <c r="D34" s="135"/>
-      <c r="E34" s="136"/>
-      <c r="F34" s="137"/>
-      <c r="G34" s="137"/>
-      <c r="H34" s="138"/>
-      <c r="I34" s="139"/>
-      <c r="J34" s="140"/>
+      <c r="B34" s="137"/>
+      <c r="C34" s="138"/>
+      <c r="D34" s="138"/>
+      <c r="E34" s="139"/>
+      <c r="F34" s="140"/>
+      <c r="G34" s="140"/>
+      <c r="H34" s="141"/>
+      <c r="I34" s="142"/>
+      <c r="J34" s="143"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>